<commit_message>
Aggiunge autoregistrazione utenti, notifiche email, conteggio difformita' confermate e rafforza scrittura SharePoint.
</commit_message>
<xml_diff>
--- a/OUTPUT_FLUSSO_CANNABIS_FINALE.xlsx
+++ b/OUTPUT_FLUSSO_CANNABIS_FINALE.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://atsinsubria.sharepoint.com/sites/IAcannabis/Archivio/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\milanif\Desktop\ats-webapp-test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="39720" documentId="8_{869A2246-5EDB-4062-B28A-714EF90C4EB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ECE58728-948B-43D8-8406-CC0766BF2FFD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF409A02-3B3A-4739-8233-CB6C4370F5CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{17CFAB25-E292-40A8-B539-58A49782BAE1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="95">
   <si>
     <t>Data_Elaborazione</t>
   </si>
@@ -300,13 +300,34 @@
   </si>
   <si>
     <t>ETICHETTA MANCANTE</t>
+  </si>
+  <si>
+    <t>LEGENDA</t>
+  </si>
+  <si>
+    <t>Difformità esclusa</t>
+  </si>
+  <si>
+    <t>Dato modificato/aggiunto</t>
+  </si>
+  <si>
+    <t>NOTE</t>
+  </si>
+  <si>
+    <t>NOTE2</t>
+  </si>
+  <si>
+    <t>NOTE3</t>
+  </si>
+  <si>
+    <t>NOTE4</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -360,8 +381,15 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="22"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -403,8 +431,32 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -412,8 +464,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="8">
+  <cellStyleXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -422,8 +489,12 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -461,9 +532,26 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="9" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="8" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="7" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="8">
+  <cellStyles count="10">
     <cellStyle name="40% - Colore 1" xfId="5" builtinId="31"/>
+    <cellStyle name="40% - Colore 4" xfId="8" builtinId="43"/>
     <cellStyle name="60% - Colore 2" xfId="3" builtinId="36"/>
     <cellStyle name="60% - Colore 3" xfId="1" builtinId="40"/>
     <cellStyle name="60% - Colore 5" xfId="7" builtinId="48"/>
@@ -471,8 +559,32 @@
     <cellStyle name="Colore 4" xfId="6" builtinId="41"/>
     <cellStyle name="Hyperlink" xfId="2" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
+    <cellStyle name="Stile 1" xfId="9" xr:uid="{B91C6F50-2D04-43D8-8277-9BF12BB075A5}"/>
   </cellStyles>
-  <dxfs count="58">
+  <dxfs count="59">
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1726,6 +1838,40 @@
       </fill>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1762,40 +1908,6 @@
       </border>
     </dxf>
     <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1838,26 +1950,6 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="left" vertical="top"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1873,7 +1965,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{71D45199-D4F5-41A2-82D6-1C5960437527}" name="Tabella_REGIONE" displayName="Tabella_REGIONE" ref="A1:AP2" insertRow="1" totalsRowShown="0" headerRowDxfId="55" headerRowCellStyle="60% - Colore 3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{71D45199-D4F5-41A2-82D6-1C5960437527}" name="Tabella_REGIONE" displayName="Tabella_REGIONE" ref="A1:AP2" insertRow="1" totalsRowShown="0" headerRowDxfId="58" headerRowCellStyle="60% - Colore 3">
   <autoFilter ref="A1:AP2" xr:uid="{71D45199-D4F5-41A2-82D6-1C5960437527}"/>
   <tableColumns count="42">
     <tableColumn id="42" xr3:uid="{63C8A22D-7BC0-44D3-82AB-6D9D79D9C7A3}" name="Data_Elaborazione"/>
@@ -1882,7 +1974,7 @@
     <tableColumn id="3" xr3:uid="{543081F9-E70A-4FF6-927A-5E7AC57F80E9}" name="FARMACIA_KEY"/>
     <tableColumn id="4" xr3:uid="{07AD7A80-DC89-4B7E-9846-0ED55BCC7255}" name="DATA_SPEDIZIONE"/>
     <tableColumn id="5" xr3:uid="{F9A04F71-0229-4DC8-AF2B-B20476A67C5C}" name="NUM_RICETTA"/>
-    <tableColumn id="6" xr3:uid="{C09B3181-35D5-4715-85CB-022999263DF1}" name="BARCODE" dataDxfId="54"/>
+    <tableColumn id="6" xr3:uid="{C09B3181-35D5-4715-85CB-022999263DF1}" name="BARCODE" dataDxfId="57"/>
     <tableColumn id="7" xr3:uid="{356F379C-4611-496F-813B-5C0CBECF7D60}" name="MEDICO_ID"/>
     <tableColumn id="8" xr3:uid="{2E3FD198-A189-4772-A414-C9C7BBD1384A}" name="ASSISTITO_ID"/>
     <tableColumn id="9" xr3:uid="{74124CB7-BE60-45E1-8DF9-BE6F66575558}" name="COD_FISCALE"/>
@@ -1924,75 +2016,88 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{506597C2-F062-49F3-9CCE-D5E3B1111146}" name="Tabella_OCR" displayName="Tabella_OCR" ref="AQ1:BO2" insertRow="1" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52" headerRowBorderDxfId="50" tableBorderDxfId="51" headerRowCellStyle="60% - Colore 3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{506597C2-F062-49F3-9CCE-D5E3B1111146}" name="Tabella_OCR" displayName="Tabella_OCR" ref="AQ1:BO2" insertRow="1" totalsRowShown="0" headerRowDxfId="56" dataDxfId="54" headerRowBorderDxfId="55" tableBorderDxfId="53" headerRowCellStyle="60% - Colore 3">
   <autoFilter ref="AQ1:BO2" xr:uid="{506597C2-F062-49F3-9CCE-D5E3B1111146}"/>
   <tableColumns count="25">
-    <tableColumn id="1" xr3:uid="{5B41D395-C6E7-4FB0-B198-7F51933DF3E1}" name="cognome_nome_assistito" dataDxfId="49"/>
-    <tableColumn id="2" xr3:uid="{D467DF96-F590-49AE-B005-8D62A9687A99}" name="barcode" dataDxfId="48"/>
-    <tableColumn id="3" xr3:uid="{A784D2AB-7A4B-43FE-ADA3-111995AF8E20}" name="codice_fiscale" dataDxfId="47"/>
-    <tableColumn id="4" xr3:uid="{57C21F6F-7080-453B-B9AC-53921EBFBFEE}" name="codice_esenzione" dataDxfId="46"/>
-    <tableColumn id="5" xr3:uid="{7C6B2D31-C987-4096-BA8C-89FE32F5A74D}" name="codice_atc" dataDxfId="45"/>
-    <tableColumn id="6" xr3:uid="{31F13015-57FB-4564-A1EF-7AB0EFBA74ED}" name="testo_prescrizione" dataDxfId="44"/>
-    <tableColumn id="7" xr3:uid="{C2983F63-DCE0-4B34-8042-8A6C02735418}" name="metodo_estrattivo_olio" dataDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{761C812B-0215-4C43-90FC-D92FB5A6BFBE}" name="forma_farmaceutica" dataDxfId="42"/>
-    <tableColumn id="9" xr3:uid="{DDFA4C58-322C-432B-8695-CF466EB0C434}" name="data_etichetta_preparazione" dataDxfId="41"/>
-    <tableColumn id="10" xr3:uid="{0C579A18-F41A-4842-92EF-2BAF9813200A}" name="data_prescrizione" dataDxfId="40"/>
-    <tableColumn id="11" xr3:uid="{E8C496A9-8C5F-4402-8C10-524BC47FEC58}" name="data_invio" dataDxfId="39"/>
-    <tableColumn id="12" xr3:uid="{BA6851C1-B9C9-4A8C-A74D-0D447792F235}" name="timbro_medico" dataDxfId="38"/>
-    <tableColumn id="13" xr3:uid="{1D7F1784-2026-43C3-BDDF-F601F025D83A}" name="firma_medico" dataDxfId="37"/>
-    <tableColumn id="14" xr3:uid="{4AA14BDE-FF9E-446D-967A-6864447358E6}" name="etichetta_avvertenze" dataDxfId="36"/>
-    <tableColumn id="15" xr3:uid="{3C37D3DD-82FD-49AF-B787-020B57269CD3}" name="etichetta_data_scadenza" dataDxfId="35"/>
-    <tableColumn id="16" xr3:uid="{0B684C51-1CED-4EA4-A871-99EC4733382F}" name="etichetta_nome_cognome_medico" dataDxfId="34"/>
-    <tableColumn id="17" xr3:uid="{D88AA7C8-90EE-423D-85FC-DDEC7F2882A8}" name="etichetta_nome_cognome_paziente" dataDxfId="33"/>
-    <tableColumn id="18" xr3:uid="{53B13049-A7FA-4093-AFD1-3F9ADDD075D4}" name="etichetta_prezzo_sost" dataDxfId="32"/>
-    <tableColumn id="19" xr3:uid="{4677C8E9-D743-4185-BF35-844262055EF6}" name="etichetta_prezzo_on" dataDxfId="31"/>
-    <tableColumn id="20" xr3:uid="{A7EB73B4-7840-4B9A-B102-5C338AB7702F}" name="etichetta_prezzo_rec" dataDxfId="30"/>
-    <tableColumn id="21" xr3:uid="{49B92581-0415-4A04-9C60-EF7E4EB82BA6}" name="etichetta_prezzo_iva" dataDxfId="29"/>
-    <tableColumn id="22" xr3:uid="{87CF3D88-874F-4462-A4BD-1066FAD0B3B9}" name="etichetta_prezzo_tot" dataDxfId="28"/>
-    <tableColumn id="23" xr3:uid="{C6D85038-F2CD-4FD8-BA6D-D84F1654FBBC}" name="totale_prescrizione" dataDxfId="27"/>
-    <tableColumn id="24" xr3:uid="{9A82A7C5-1920-437E-A807-97B749A9402B}" name="etichetta_THC" dataDxfId="26"/>
-    <tableColumn id="25" xr3:uid="{20CAA407-BFB4-4AC9-B25A-CA009247E627}" name="nome_farmacia" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{5B41D395-C6E7-4FB0-B198-7F51933DF3E1}" name="cognome_nome_assistito" dataDxfId="52"/>
+    <tableColumn id="2" xr3:uid="{D467DF96-F590-49AE-B005-8D62A9687A99}" name="barcode" dataDxfId="51"/>
+    <tableColumn id="3" xr3:uid="{A784D2AB-7A4B-43FE-ADA3-111995AF8E20}" name="codice_fiscale" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{57C21F6F-7080-453B-B9AC-53921EBFBFEE}" name="codice_esenzione" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{7C6B2D31-C987-4096-BA8C-89FE32F5A74D}" name="codice_atc" dataDxfId="48"/>
+    <tableColumn id="6" xr3:uid="{31F13015-57FB-4564-A1EF-7AB0EFBA74ED}" name="testo_prescrizione" dataDxfId="47"/>
+    <tableColumn id="7" xr3:uid="{C2983F63-DCE0-4B34-8042-8A6C02735418}" name="metodo_estrattivo_olio" dataDxfId="46"/>
+    <tableColumn id="8" xr3:uid="{761C812B-0215-4C43-90FC-D92FB5A6BFBE}" name="forma_farmaceutica" dataDxfId="45"/>
+    <tableColumn id="9" xr3:uid="{DDFA4C58-322C-432B-8695-CF466EB0C434}" name="data_etichetta_preparazione" dataDxfId="44"/>
+    <tableColumn id="10" xr3:uid="{0C579A18-F41A-4842-92EF-2BAF9813200A}" name="data_prescrizione" dataDxfId="43"/>
+    <tableColumn id="11" xr3:uid="{E8C496A9-8C5F-4402-8C10-524BC47FEC58}" name="data_invio" dataDxfId="42"/>
+    <tableColumn id="12" xr3:uid="{BA6851C1-B9C9-4A8C-A74D-0D447792F235}" name="timbro_medico" dataDxfId="41"/>
+    <tableColumn id="13" xr3:uid="{1D7F1784-2026-43C3-BDDF-F601F025D83A}" name="firma_medico" dataDxfId="40"/>
+    <tableColumn id="14" xr3:uid="{4AA14BDE-FF9E-446D-967A-6864447358E6}" name="etichetta_avvertenze" dataDxfId="39"/>
+    <tableColumn id="15" xr3:uid="{3C37D3DD-82FD-49AF-B787-020B57269CD3}" name="etichetta_data_scadenza" dataDxfId="38"/>
+    <tableColumn id="16" xr3:uid="{0B684C51-1CED-4EA4-A871-99EC4733382F}" name="etichetta_nome_cognome_medico" dataDxfId="37"/>
+    <tableColumn id="17" xr3:uid="{D88AA7C8-90EE-423D-85FC-DDEC7F2882A8}" name="etichetta_nome_cognome_paziente" dataDxfId="36"/>
+    <tableColumn id="18" xr3:uid="{53B13049-A7FA-4093-AFD1-3F9ADDD075D4}" name="etichetta_prezzo_sost" dataDxfId="35"/>
+    <tableColumn id="19" xr3:uid="{4677C8E9-D743-4185-BF35-844262055EF6}" name="etichetta_prezzo_on" dataDxfId="34"/>
+    <tableColumn id="20" xr3:uid="{A7EB73B4-7840-4B9A-B102-5C338AB7702F}" name="etichetta_prezzo_rec" dataDxfId="33"/>
+    <tableColumn id="21" xr3:uid="{49B92581-0415-4A04-9C60-EF7E4EB82BA6}" name="etichetta_prezzo_iva" dataDxfId="32"/>
+    <tableColumn id="22" xr3:uid="{87CF3D88-874F-4462-A4BD-1066FAD0B3B9}" name="etichetta_prezzo_tot" dataDxfId="31"/>
+    <tableColumn id="23" xr3:uid="{C6D85038-F2CD-4FD8-BA6D-D84F1654FBBC}" name="totale_prescrizione" dataDxfId="30"/>
+    <tableColumn id="24" xr3:uid="{9A82A7C5-1920-437E-A807-97B749A9402B}" name="etichetta_THC" dataDxfId="29"/>
+    <tableColumn id="25" xr3:uid="{20CAA407-BFB4-4AC9-B25A-CA009247E627}" name="nome_farmacia" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{DEF5942A-0AC7-4697-BACB-DB14AB0DC041}" name="Tabella_LINK" displayName="Tabella_LINK" ref="BP1:BP2" insertRow="1" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23" headerRowCellStyle="60% - Colore 3" dataCellStyle="60% - Colore 3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{DEF5942A-0AC7-4697-BACB-DB14AB0DC041}" name="Tabella_LINK" displayName="Tabella_LINK" ref="BP1:BP2" insertRow="1" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26" headerRowCellStyle="60% - Colore 3" dataCellStyle="60% - Colore 3">
   <autoFilter ref="BP1:BP2" xr:uid="{DEF5942A-0AC7-4697-BACB-DB14AB0DC041}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{BD66DB9A-5E0A-4504-A937-48D92A9EBF0B}" name="LINK" dataDxfId="22" dataCellStyle="60% - Colore 3"/>
+    <tableColumn id="1" xr3:uid="{BD66DB9A-5E0A-4504-A937-48D92A9EBF0B}" name="LINK" dataDxfId="25" dataCellStyle="60% - Colore 3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6D7E05F9-AC03-4073-9B73-9181FC532C87}" name="Tabella_LLM" displayName="Tabella_LLM" ref="BQ1:CJ2" insertRow="1" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6D7E05F9-AC03-4073-9B73-9181FC532C87}" name="Tabella_LLM" displayName="Tabella_LLM" ref="BQ1:CJ2" insertRow="1" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
   <autoFilter ref="BQ1:CJ2" xr:uid="{6D7E05F9-AC03-4073-9B73-9181FC532C87}"/>
   <tableColumns count="20">
-    <tableColumn id="2" xr3:uid="{7B60B60E-CB98-41CB-A0B0-B2E37D5026A2}" name="R02" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{D6A456B8-46A2-49E5-8CA4-1B6B4DEFF20C}" name="R03" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{6A889835-BCE7-4F69-9D35-8E1F84DD7360}" name="R04" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{3905CAE4-6AEA-40DC-87BA-C3EF2857AC95}" name="R05" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{3B5A9286-39FF-43C4-B9DC-E2B0891BDCA9}" name="R07" dataDxfId="15"/>
-    <tableColumn id="7" xr3:uid="{2368315B-771A-4583-9A05-8643C2903FF0}" name="R05A" dataDxfId="14"/>
-    <tableColumn id="8" xr3:uid="{816B82D3-C621-4E06-9195-08BADC6CE0B0}" name="R06" dataDxfId="13"/>
-    <tableColumn id="9" xr3:uid="{4DFEAC33-18A7-45FF-B1B0-F5F68390935F}" name="R08" dataDxfId="12"/>
-    <tableColumn id="10" xr3:uid="{39E4656E-7D12-4F23-AE2A-C2E879F052D4}" name="R09" dataDxfId="11"/>
-    <tableColumn id="11" xr3:uid="{157023CB-2F73-44B4-8A68-8A9E92848FAE}" name="R10" dataDxfId="10"/>
-    <tableColumn id="20" xr3:uid="{16C3FEEC-7118-49A6-BCB8-77EE3EC9EE3B}" name="R10A" dataDxfId="9"/>
-    <tableColumn id="12" xr3:uid="{FC89075B-0669-4F16-9C3F-96B543D1FBC1}" name="R01" dataDxfId="8"/>
-    <tableColumn id="13" xr3:uid="{6DD4ECE4-F620-4A53-85DE-DFC219F78826}" name="R11" dataDxfId="7"/>
-    <tableColumn id="14" xr3:uid="{380F4E21-85E6-4ED2-8836-7A77624B4867}" name="R12" dataDxfId="6"/>
-    <tableColumn id="15" xr3:uid="{887EA67A-C4B9-4143-AF6F-A0D247E107F4}" name="R13" dataDxfId="5"/>
-    <tableColumn id="16" xr3:uid="{A8242F01-6A27-4B06-8650-0CDCC24F994C}" name="R16" dataDxfId="4"/>
-    <tableColumn id="17" xr3:uid="{616E93F8-4A12-4269-A156-6ECFCC3C542C}" name="R19" dataDxfId="3"/>
-    <tableColumn id="18" xr3:uid="{D2607DCA-98F3-47CA-AA3A-1BA350614801}" name="R14" dataDxfId="2"/>
-    <tableColumn id="19" xr3:uid="{0788E116-AC43-463D-A122-0C96ECB41612}" name="R18" dataDxfId="1"/>
-    <tableColumn id="21" xr3:uid="{B758F35A-48E7-458B-8385-F294CB3F3457}" name="ETICHETTA MANCANTE" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{7B60B60E-CB98-41CB-A0B0-B2E37D5026A2}" name="R02" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{D6A456B8-46A2-49E5-8CA4-1B6B4DEFF20C}" name="R03" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{6A889835-BCE7-4F69-9D35-8E1F84DD7360}" name="R04" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{3905CAE4-6AEA-40DC-87BA-C3EF2857AC95}" name="R05" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{3B5A9286-39FF-43C4-B9DC-E2B0891BDCA9}" name="R07" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{2368315B-771A-4583-9A05-8643C2903FF0}" name="R05A" dataDxfId="17"/>
+    <tableColumn id="8" xr3:uid="{816B82D3-C621-4E06-9195-08BADC6CE0B0}" name="R06" dataDxfId="16"/>
+    <tableColumn id="9" xr3:uid="{4DFEAC33-18A7-45FF-B1B0-F5F68390935F}" name="R08" dataDxfId="15"/>
+    <tableColumn id="10" xr3:uid="{39E4656E-7D12-4F23-AE2A-C2E879F052D4}" name="R09" dataDxfId="14"/>
+    <tableColumn id="11" xr3:uid="{157023CB-2F73-44B4-8A68-8A9E92848FAE}" name="R10" dataDxfId="13"/>
+    <tableColumn id="20" xr3:uid="{16C3FEEC-7118-49A6-BCB8-77EE3EC9EE3B}" name="R10A" dataDxfId="12"/>
+    <tableColumn id="12" xr3:uid="{FC89075B-0669-4F16-9C3F-96B543D1FBC1}" name="R01" dataDxfId="11"/>
+    <tableColumn id="13" xr3:uid="{6DD4ECE4-F620-4A53-85DE-DFC219F78826}" name="R11" dataDxfId="10"/>
+    <tableColumn id="14" xr3:uid="{380F4E21-85E6-4ED2-8836-7A77624B4867}" name="R12" dataDxfId="9"/>
+    <tableColumn id="15" xr3:uid="{887EA67A-C4B9-4143-AF6F-A0D247E107F4}" name="R13" dataDxfId="8"/>
+    <tableColumn id="16" xr3:uid="{A8242F01-6A27-4B06-8650-0CDCC24F994C}" name="R16" dataDxfId="7"/>
+    <tableColumn id="17" xr3:uid="{616E93F8-4A12-4269-A156-6ECFCC3C542C}" name="R19" dataDxfId="6"/>
+    <tableColumn id="18" xr3:uid="{D2607DCA-98F3-47CA-AA3A-1BA350614801}" name="R14" dataDxfId="5"/>
+    <tableColumn id="19" xr3:uid="{0788E116-AC43-463D-A122-0C96ECB41612}" name="R18" dataDxfId="4"/>
+    <tableColumn id="21" xr3:uid="{B758F35A-48E7-458B-8385-F294CB3F3457}" name="ETICHETTA MANCANTE" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{972D6864-75FD-486B-AE17-DDF79BFEAB7B}" name="Tabella5" displayName="Tabella5" ref="CK1:CN1048576" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="CK1:CN1048576" xr:uid="{972D6864-75FD-486B-AE17-DDF79BFEAB7B}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{4FA6D3C5-7805-407B-A60F-D32D8C73AA99}" name="NOTE"/>
+    <tableColumn id="2" xr3:uid="{ACAEBE43-D941-49EA-AEFB-90F3F7CBB798}" name="NOTE2"/>
+    <tableColumn id="3" xr3:uid="{DC553359-E62A-4D7E-8082-34ADF8395F75}" name="NOTE3"/>
+    <tableColumn id="4" xr3:uid="{CE0EF4D5-EE27-4B48-AAC2-7AA6ADAC7184}" name="NOTE4"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -2313,8 +2418,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F8AAD1F-E170-47FA-AF9E-FC31CC74C2CE}">
-  <dimension ref="A1:CJ37"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:CR37"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="43.7109375" bestFit="1" customWidth="1"/>
@@ -2398,9 +2503,14 @@
     <col min="86" max="86" width="26.140625" bestFit="1" customWidth="1"/>
     <col min="87" max="87" width="37.7109375" customWidth="1"/>
     <col min="88" max="88" width="27.7109375" customWidth="1"/>
+    <col min="89" max="89" width="21.7109375" customWidth="1"/>
+    <col min="90" max="90" width="16" customWidth="1"/>
+    <col min="91" max="91" width="19.42578125" customWidth="1"/>
+    <col min="92" max="92" width="10.7109375" customWidth="1"/>
+    <col min="96" max="96" width="17.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:88" s="5" customFormat="1">
+    <row r="1" spans="1:96" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2665,8 +2775,24 @@
       <c r="CJ1" s="13" t="s">
         <v>87</v>
       </c>
+      <c r="CK1" s="28" t="s">
+        <v>91</v>
+      </c>
+      <c r="CL1" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="CM1" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="CN1" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="CQ1" s="26" t="s">
+        <v>88</v>
+      </c>
+      <c r="CR1" s="27"/>
     </row>
-    <row r="2" spans="1:88" ht="21.75" customHeight="1">
+    <row r="2" spans="1:96" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2748,54 +2874,95 @@
       <c r="CH2" s="20"/>
       <c r="CI2" s="20"/>
       <c r="CJ2" s="21"/>
+      <c r="CK2" s="21"/>
+      <c r="CQ2" s="27"/>
+      <c r="CR2" s="27"/>
     </row>
-    <row r="22" spans="9:9" ht="18" customHeight="1"/>
-    <row r="27" spans="9:9" ht="15" customHeight="1">
+    <row r="3" spans="1:96" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="CQ3" s="27"/>
+      <c r="CR3" s="27"/>
+    </row>
+    <row r="4" spans="1:96" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="CQ4" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="CR4" s="24"/>
+    </row>
+    <row r="5" spans="1:96" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="CQ5" s="25" t="s">
+        <v>90</v>
+      </c>
+      <c r="CR5" s="25"/>
+    </row>
+    <row r="6" spans="1:96" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="CM6" s="23"/>
+      <c r="CN6" s="23"/>
+    </row>
+    <row r="7" spans="1:96" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="CM7" s="23"/>
+      <c r="CN7" s="23"/>
+    </row>
+    <row r="8" spans="1:96" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="CM8" s="23"/>
+      <c r="CN8" s="23"/>
+    </row>
+    <row r="9" spans="1:96" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="CM9" s="23"/>
+      <c r="CN9" s="23"/>
+    </row>
+    <row r="22" spans="9:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="9:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I27" s="1"/>
     </row>
-    <row r="28" spans="9:9" ht="15" customHeight="1">
+    <row r="28" spans="9:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I28" s="1"/>
     </row>
-    <row r="29" spans="9:9" ht="15" customHeight="1">
+    <row r="29" spans="9:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I29" s="1"/>
     </row>
-    <row r="30" spans="9:9" ht="15" customHeight="1">
+    <row r="30" spans="9:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I30" s="1"/>
     </row>
-    <row r="31" spans="9:9" ht="15" customHeight="1">
+    <row r="31" spans="9:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I31" s="1"/>
     </row>
-    <row r="32" spans="9:9" ht="15" customHeight="1">
+    <row r="32" spans="9:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I32" s="1"/>
     </row>
-    <row r="33" spans="9:9" ht="15" customHeight="1">
+    <row r="33" spans="9:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I33" s="1"/>
     </row>
-    <row r="34" spans="9:9" ht="15" customHeight="1">
+    <row r="34" spans="9:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I34" s="1"/>
     </row>
-    <row r="35" spans="9:9" ht="15" customHeight="1">
+    <row r="35" spans="9:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I35" s="1"/>
     </row>
-    <row r="36" spans="9:9" ht="15" customHeight="1">
+    <row r="36" spans="9:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I36" s="1"/>
     </row>
-    <row r="37" spans="9:9" ht="15" customHeight="1">
+    <row r="37" spans="9:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I37" s="1"/>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="CQ4:CR4"/>
+    <mergeCell ref="CQ5:CR5"/>
+    <mergeCell ref="CQ1:CR3"/>
+  </mergeCells>
   <conditionalFormatting sqref="G3:G1048576 G1">
-    <cfRule type="duplicateValues" dxfId="57" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="AR3:AR1048576 AR1">
-    <cfRule type="duplicateValues" dxfId="56" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="4">
+  <tableParts count="5">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2977,17 +3144,45 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A623CC41-114C-4059-97DA-9B9775C6BEC4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A623CC41-114C-4059-97DA-9B9775C6BEC4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5176c8bf-9894-4624-8291-6a05c0973339"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2AAA7497-FDBD-4CCD-9FA7-75732EC779ED}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2AAA7497-FDBD-4CCD-9FA7-75732EC779ED}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/extensibility/maker/v1.0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3EC2676D-1EB0-4099-92E4-18213106A7C9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3EC2676D-1EB0-4099-92E4-18213106A7C9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5176c8bf-9894-4624-8291-6a05c0973339"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D967F51-13D8-4180-A954-27E447B85CC4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D967F51-13D8-4180-A954-27E447B85CC4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>